<commit_message>
Add RS_CFG_EN parameter verification
</commit_message>
<xml_diff>
--- a/examples/RS_Check_Excel_Template.xlsx
+++ b/examples/RS_Check_Excel_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="R68726103f93b4c69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R8eeb67a13da7452b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="Rcb0ce2d5b6fe487e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="Rd18c6586786241be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -135,7 +135,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="44">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -231,6 +231,21 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -240,9 +255,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RSCheckInputTable" displayName="RSCheckInputTable" ref="A1:H3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H3"/>
-  <x:tableColumns count="8">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RSCheckInputTable" displayName="RSCheckInputTable" ref="A1:I3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
     <x:tableColumn id="1" name="Intf_type"/>
     <x:tableColumn id="2" name="RS_module"/>
     <x:tableColumn id="3" name="RS_inst"/>
@@ -251,13 +265,14 @@
     <x:tableColumn id="6" name="clk"/>
     <x:tableColumn id="7" name="rst"/>
     <x:tableColumn id="8" name="CRG_source"/>
+    <x:tableColumn id="9" name="RS_CFG_EN"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RSCheckFieldGuideTable" displayName="RSCheckFieldGuideTable" ref="A5:G13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RSCheckFieldGuideTable" displayName="RSCheckFieldGuideTable" ref="A5:G14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="默认列"/>
     <x:tableColumn id="2" name="字段"/>
@@ -474,6 +489,7 @@
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -501,6 +517,9 @@
       <x:c r="H1" s="5" t="str">
         <x:v>CRG_source</x:v>
       </x:c>
+      <x:c r="I1" s="44" t="str">
+        <x:v>RS_CFG_EN</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -527,6 +546,9 @@
       <x:c r="H2" s="9" t="str">
         <x:v>crg_core</x:v>
       </x:c>
+      <x:c r="I2" t="str">
+        <x:v>假门控</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="9" t="str">
@@ -553,17 +575,23 @@
       <x:c r="H3" s="9" t="str">
         <x:v>crg_aux</x:v>
       </x:c>
+      <x:c r="I3" t="str">
+        <x:v>假门控</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="whole" operator="between" sqref="E2:E3">
       <x:formula1>1</x:formula1>
       <x:formula2>2147483647</x:formula2>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="I2:I3">
+      <x:formula1>"假门控"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfd1a69a05224277"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9921415e2514523"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -654,7 +682,7 @@
         <x:v>OUT_IF</x:v>
       </x:c>
       <x:c r="F6" s="33" t="str">
-        <x:v>v1 仅写入报告，不参与通过/失败判定</x:v>
+        <x:v>当前仅写入报告，不参与通过/失败判定</x:v>
       </x:c>
       <x:c r="G6" s="33" t="str">
         <x:v>不可留空</x:v>
@@ -819,6 +847,29 @@
       </x:c>
       <x:c r="G13" s="33" t="str">
         <x:v>多驱动或无法解析来源时检查失败</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="56" customHeight="1">
+      <x:c r="A14" s="48" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="B14" s="48" t="str">
+        <x:v>RS_CFG_EN</x:v>
+      </x:c>
+      <x:c r="C14" s="48" t="str">
+        <x:v>条件必填 / 文本</x:v>
+      </x:c>
+      <x:c r="D14" s="47" t="str">
+        <x:v>RTL 模块具有同名参数时的假门控标记</x:v>
+      </x:c>
+      <x:c r="E14" s="47" t="str">
+        <x:v>假门控</x:v>
+      </x:c>
+      <x:c r="F14" s="47" t="str">
+        <x:v>逐实例读取 elaboration 后值；仅参数为 0 且本列为假门控时通过</x:v>
+      </x:c>
+      <x:c r="G14" s="47" t="str">
+        <x:v>参数不存在时留空；参数存在时必须填假门控</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
@@ -877,7 +928,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb6ca565f57e4d20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re237ef7e777e4f9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add module rule driven dynamic step checks
</commit_message>
<xml_diff>
--- a/examples/RS_Check_Excel_Template.xlsx
+++ b/examples/RS_Check_Excel_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="Rcb0ce2d5b6fe487e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="Rd18c6586786241be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="R9c1d0055713d41d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="Rce3c81a31acf49af"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -68,7 +68,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -88,6 +88,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7F9FC"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -135,7 +145,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="49">
+  <x:cellXfs count="59">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -246,6 +256,26 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -535,7 +565,7 @@
         <x:v>top.u_tile</x:v>
       </x:c>
       <x:c r="E2" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
         <x:v>clk_rs</x:v>
@@ -582,7 +612,7 @@
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="whole" operator="between" sqref="E2:E3">
-      <x:formula1>1</x:formula1>
+      <x:formula1>0</x:formula1>
       <x:formula2>2147483647</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I2:I3">
@@ -591,7 +621,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9921415e2514523"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43370e4ae05b4a15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -705,10 +735,10 @@
         <x:v>rs_pipe</x:v>
       </x:c>
       <x:c r="F7" s="33" t="str">
-        <x:v>与实例的 NPI npiDefName 精确比较</x:v>
+        <x:v>先匹配模块规则库，再与实例的 NPI npiDefName 精确比较</x:v>
       </x:c>
       <x:c r="G7" s="33" t="str">
-        <x:v>填写模块名，不是例化名</x:v>
+        <x:v>必须先在 GUI 模块规则库或 config.module_rules 中登记</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
@@ -765,19 +795,19 @@
         <x:v>step</x:v>
       </x:c>
       <x:c r="C10" s="32" t="str">
-        <x:v>是 / 正整数</x:v>
+        <x:v>是 / 非负整数</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
-        <x:v>当前 position 下该实例组的总打拍数</x:v>
+        <x:v>当前 position 下该实例组的有效总打拍数</x:v>
       </x:c>
       <x:c r="E10" s="33" t="str">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F10" s="33" t="str">
-        <x:v>有效组成员数量必须等于 step</x:v>
+        <x:v>按模块规则逐实例计算 0/1 贡献，贡献和必须等于 step</x:v>
       </x:c>
       <x:c r="G10" s="33" t="str">
-        <x:v>每个有效例化计 1 拍，最小值为 1</x:v>
+        <x:v>控制参数为 0 的实例贡献 0；全部关闭时可填 0</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -860,16 +890,16 @@
         <x:v>条件必填 / 文本</x:v>
       </x:c>
       <x:c r="D14" s="47" t="str">
-        <x:v>RTL 模块具有同名参数时的假门控标记</x:v>
+        <x:v>模块规则声明有同名参数时的假门控标记</x:v>
       </x:c>
       <x:c r="E14" s="47" t="str">
         <x:v>假门控</x:v>
       </x:c>
       <x:c r="F14" s="47" t="str">
-        <x:v>逐实例读取 elaboration 后值；仅参数为 0 且本列为假门控时通过</x:v>
+        <x:v>按模块规则逐实例检查存在性；参数值为 0 且本列为假门控时通过</x:v>
       </x:c>
       <x:c r="G14" s="47" t="str">
-        <x:v>参数不存在时留空；参数存在时必须填假门控</x:v>
+        <x:v>规则声明无参数时留空；声明有参数时必须填假门控</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
@@ -915,6 +945,39 @@
       <x:c r="E18" s="43"/>
       <x:c r="F18" s="43"/>
       <x:c r="G18" s="43"/>
+    </x:row>
+    <x:row r="19" ht="26" customHeight="1">
+      <x:c r="A19" s="52" t="str">
+        <x:v>模块规则库与有效拍数规则</x:v>
+      </x:c>
+      <x:c r="B19" s="52"/>
+      <x:c r="C19" s="52"/>
+      <x:c r="D19" s="52"/>
+      <x:c r="E19" s="52"/>
+      <x:c r="F19" s="52"/>
+      <x:c r="G19" s="52"/>
+    </x:row>
+    <x:row r="20" ht="34" customHeight="1">
+      <x:c r="A20" s="58" t="str">
+        <x:v>每个 RS_module 必须在 config.module_rules 登记 has_rs_cfg_en 和 step_parameters；Excel 模块名按大小写精确匹配。</x:v>
+      </x:c>
+      <x:c r="B20" s="58"/>
+      <x:c r="C20" s="58"/>
+      <x:c r="D20" s="58"/>
+      <x:c r="E20" s="58"/>
+      <x:c r="F20" s="58"/>
+      <x:c r="G20" s="58"/>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="58" t="str">
+        <x:v>每个物理实例的全部 step_parameters 均非零时贡献 1，任一为 0 时贡献 0；缺失、X/Z 或无法解析时检查失败。</x:v>
+      </x:c>
+      <x:c r="B21" s="58"/>
+      <x:c r="C21" s="58"/>
+      <x:c r="D21" s="58"/>
+      <x:c r="E21" s="58"/>
+      <x:c r="F21" s="58"/>
+      <x:c r="G21" s="58"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -925,10 +988,13 @@
     <x:mergeCell ref="A16:G16"/>
     <x:mergeCell ref="A17:G17"/>
     <x:mergeCell ref="A18:G18"/>
+    <x:mergeCell ref="A19:G19"/>
+    <x:mergeCell ref="A20:G20"/>
+    <x:mergeCell ref="A21:G21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re237ef7e777e4f9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65a24f194f8f4b60"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add position alias mapping database
</commit_message>
<xml_diff>
--- a/examples/RS_Check_Excel_Template.xlsx
+++ b/examples/RS_Check_Excel_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="R9c1d0055713d41d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="Rce3c81a31acf49af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="Raad73ca9a9424b8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R8edf3f066d9049a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -562,7 +562,7 @@
         <x:v>AAAA_BBB</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>top.u_tile</x:v>
+        <x:v>tile_core</x:v>
       </x:c>
       <x:c r="E2" s="11" t="n">
         <x:v>5</x:v>
@@ -591,7 +591,7 @@
         <x:v>CTRL_RS</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>top.u_tile</x:v>
+        <x:v>tile_core</x:v>
       </x:c>
       <x:c r="E3" s="11" t="n">
         <x:v>1</x:v>
@@ -621,7 +621,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43370e4ae05b4a15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98313216a26e4bbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -652,7 +652,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="19" t="str">
-        <x:v>一行定义一个实例组，唯一键为 (position, RS_inst)。RS_Check 第 2-3 行为示例，请替换后使用。</x:v>
+        <x:v>一行定义一个实例组，唯一键为解析后全路径对应的 (position, RS_inst)。RS_Check 第 2-3 行为示例，请替换后使用。</x:v>
       </x:c>
       <x:c r="B2" s="19"/>
       <x:c r="C2" s="19"/>
@@ -738,7 +738,7 @@
         <x:v>先匹配模块规则库，再与实例的 NPI npiDefName 精确比较</x:v>
       </x:c>
       <x:c r="G7" s="33" t="str">
-        <x:v>必须先在 GUI 模块规则库或 config.module_rules 中登记</x:v>
+        <x:v>未登记模块使用默认规则；仅在需要覆盖默认行为时添加显式规则</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
@@ -775,16 +775,16 @@
         <x:v>是 / 文本</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
-        <x:v>该组实例直接父 scope 的完整 NPI 层级路径</x:v>
+        <x:v>该组实例直接父 scope 的 position 简写或完整 NPI 层级路径</x:v>
       </x:c>
       <x:c r="E9" s="33" t="str">
-        <x:v>top.u_tile</x:v>
+        <x:v>tile_core</x:v>
       </x:c>
       <x:c r="F9" s="33" t="str">
-        <x:v>在此 scope 下查找 RS_inst 组成员</x:v>
+        <x:v>先按 config.position_mappings 精确解析，再在全路径 scope 下查找</x:v>
       </x:c>
       <x:c r="G9" s="33" t="str">
-        <x:v>不要填到具体打拍实例本身</x:v>
+        <x:v>简写需在 GUI Position映射库登记；未命中时按完整路径使用</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -904,7 +904,7 @@
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
       <x:c r="A15" s="37" t="str">
-        <x:v>分组与列映射规则</x:v>
+        <x:v>分组、Position映射与列映射规则</x:v>
       </x:c>
       <x:c r="B15" s="37"/>
       <x:c r="C15" s="37"/>
@@ -926,7 +926,7 @@
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="43" t="str">
-        <x:v>同一个 position 可以有多个组，每组占一行；同一 (position, RS_inst) 组合不能重复。</x:v>
+        <x:v>position 可填简写；config.position_mappings 存在同名 key 时解析为对应 RTL 全路径，未命中则兼容原有完整路径。</x:v>
       </x:c>
       <x:c r="B17" s="43"/>
       <x:c r="C17" s="43"/>
@@ -959,7 +959,7 @@
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
       <x:c r="A20" s="58" t="str">
-        <x:v>每个 RS_module 必须在 config.module_rules 登记 has_rs_cfg_en 和 step_parameters；Excel 模块名按大小写精确匹配。</x:v>
+        <x:v>未登记 RS_module 使用默认 has_rs_cfg_en=true、step_parameters=[]；大小写精确匹配的显式规则优先。</x:v>
       </x:c>
       <x:c r="B20" s="58"/>
       <x:c r="C20" s="58"/>
@@ -994,7 +994,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65a24f194f8f4b60"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27678fb9d703493d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Allow complete RS instance names
</commit_message>
<xml_diff>
--- a/examples/RS_Check_Excel_Template.xlsx
+++ b/examples/RS_Check_Excel_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="Raad73ca9a9424b8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R8edf3f066d9049a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="Rcb6dca023ff84fcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="Rbaa40f273653467c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -588,7 +588,7 @@
         <x:v>rs_pipe</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>CTRL_RS</x:v>
+        <x:v>CTRL_RS_D0</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
         <x:v>tile_core</x:v>
@@ -621,7 +621,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98313216a26e4bbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re904c03b801644c8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -752,16 +752,16 @@
         <x:v>是 / 文本</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
-        <x:v>组内本地例化名的共同前缀</x:v>
+        <x:v>组内本地例化名的共同前缀，或完整本地例化名</x:v>
       </x:c>
       <x:c r="E8" s="33" t="str">
-        <x:v>AAAA_BBB</x:v>
+        <x:v>AAAA_BBB / CTRL_RS_D0</x:v>
       </x:c>
       <x:c r="F8" s="33" t="str">
-        <x:v>匹配此前缀，并校验其余后缀符合 suffix_regex</x:v>
+        <x:v>空后缀直接匹配；非空后缀按 suffix_regex 校验</x:v>
       </x:c>
       <x:c r="G8" s="33" t="str">
-        <x:v>例如匹配 AAAA_BBB_C0、AAAA_BBB_C1</x:v>
+        <x:v>RS_inst 本身不可为空；不要填写 position.RS_inst 层次全路径</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -915,7 +915,7 @@
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
       <x:c r="A16" s="43" t="str">
-        <x:v>RS_inst=AAAA_BBB 时，可匹配 AAAA_BBB_C0、AAAA_BBB_C1；剩余后缀 _C0 / _C1 需满足 config.rtl.suffix_regex。</x:v>
+        <x:v>RS_inst=CTRL_RS_D0 时可直接匹配同名本地实例（空后缀）；RS_inst=AAAA_BBB 时可匹配 AAAA_BBB_C0、AAAA_BBB_C1，非空后缀仍需满足 config.rtl.suffix_regex。</x:v>
       </x:c>
       <x:c r="B16" s="43"/>
       <x:c r="C16" s="43"/>
@@ -994,7 +994,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27678fb9d703493d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe258f594a76457a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Allow Excel headers independent of field mappings
</commit_message>
<xml_diff>
--- a/examples/RS_Check_Excel_Template.xlsx
+++ b/examples/RS_Check_Excel_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="Rcb6dca023ff84fcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="Rbaa40f273653467c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="R15a2231bff474375"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R78e05676c95741dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -285,27 +285,29 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RSCheckInputTable" displayName="RSCheckInputTable" ref="A1:I3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RSCheckInputTable" displayName="RSCheckInputTable" ref="A1:I3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I3"/>
   <x:tableColumns count="9">
-    <x:tableColumn id="1" name="Intf_type"/>
-    <x:tableColumn id="2" name="RS_module"/>
-    <x:tableColumn id="3" name="RS_inst"/>
-    <x:tableColumn id="4" name="position"/>
-    <x:tableColumn id="5" name="step"/>
-    <x:tableColumn id="6" name="clk"/>
-    <x:tableColumn id="7" name="rst"/>
-    <x:tableColumn id="8" name="CRG_source"/>
-    <x:tableColumn id="9" name="RS_CFG_EN"/>
+    <x:tableColumn id="1" name="接口分类"/>
+    <x:tableColumn id="2" name="模块类型"/>
+    <x:tableColumn id="3" name="实例组"/>
+    <x:tableColumn id="4" name="位置简称"/>
+    <x:tableColumn id="5" name="有效拍数"/>
+    <x:tableColumn id="6" name="时钟连接"/>
+    <x:tableColumn id="7" name="复位连接"/>
+    <x:tableColumn id="8" name="时钟源模块"/>
+    <x:tableColumn id="9" name="假门控标记"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RSCheckFieldGuideTable" displayName="RSCheckFieldGuideTable" ref="A5:G14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="RSCheckFieldGuideTable" displayName="RSCheckFieldGuideTable" ref="A5:G14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:G14"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="默认列"/>
-    <x:tableColumn id="2" name="字段"/>
+    <x:tableColumn id="2" name="工具内部属性"/>
     <x:tableColumn id="3" name="必填 / 类型"/>
     <x:tableColumn id="4" name="含义"/>
     <x:tableColumn id="5" name="示例"/>
@@ -524,31 +526,31 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>Intf_type</x:v>
+        <x:v>接口分类</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str">
-        <x:v>RS_module</x:v>
+        <x:v>模块类型</x:v>
       </x:c>
       <x:c r="C1" s="5" t="str">
-        <x:v>RS_inst</x:v>
+        <x:v>实例组</x:v>
       </x:c>
       <x:c r="D1" s="5" t="str">
-        <x:v>position</x:v>
+        <x:v>位置简称</x:v>
       </x:c>
       <x:c r="E1" s="5" t="str">
-        <x:v>step</x:v>
+        <x:v>有效拍数</x:v>
       </x:c>
       <x:c r="F1" s="5" t="str">
-        <x:v>clk</x:v>
+        <x:v>时钟连接</x:v>
       </x:c>
       <x:c r="G1" s="5" t="str">
-        <x:v>rst</x:v>
+        <x:v>复位连接</x:v>
       </x:c>
       <x:c r="H1" s="5" t="str">
-        <x:v>CRG_source</x:v>
+        <x:v>时钟源模块</x:v>
       </x:c>
       <x:c r="I1" s="44" t="str">
-        <x:v>RS_CFG_EN</x:v>
+        <x:v>假门控标记</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
@@ -621,7 +623,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re904c03b801644c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88d3814b374b4dce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -663,7 +665,7 @@
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="24" t="str">
-        <x:v>默认列可以调整，但必须同步修改 config 中的 1-based columns 映射；映射字段必须使用精确表头，且不能填写公式。</x:v>
+        <x:v>列号映射决定字段归属；实际表头文字可以任意。Intf_type 等名称只是工具内部属性，只有主动启用严格表头校验时才要求同名。</x:v>
       </x:c>
       <x:c r="B3" s="24"/>
       <x:c r="C3" s="24"/>
@@ -677,7 +679,7 @@
         <x:v>默认列</x:v>
       </x:c>
       <x:c r="B5" s="29" t="str">
-        <x:v>字段</x:v>
+        <x:v>工具内部属性</x:v>
       </x:c>
       <x:c r="C5" s="29" t="str">
         <x:v>必填 / 类型</x:v>
@@ -937,7 +939,7 @@
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
       <x:c r="A18" s="43" t="str">
-        <x:v>若调整字段顺序或插入无关列，请同步修改 config/rscheck.example.json 的 columns；列号从 1 开始。</x:v>
+        <x:v>若调整字段顺序或插入无关列，请同步修改 config/rscheck.example.json 的 columns；列号从 1 开始。重命名表头无需修改映射。</x:v>
       </x:c>
       <x:c r="B18" s="43"/>
       <x:c r="C18" s="43"/>
@@ -994,7 +996,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe258f594a76457a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a9afd08293f4e57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Ignore RS_CFG_EN labels for modules without gating
</commit_message>
<xml_diff>
--- a/examples/RS_Check_Excel_Template.xlsx
+++ b/examples/RS_Check_Excel_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="R15a2231bff474375"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R78e05676c95741dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="R5184ee48631e4f5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R3e19f890b83a48b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -612,18 +612,15 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="1">
     <x:dataValidation type="whole" operator="between" sqref="E2:E3">
       <x:formula1>0</x:formula1>
       <x:formula2>2147483647</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I2:I3">
-      <x:formula1>"假门控"</x:formula1>
-    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88d3814b374b4dce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a190cfa1a144a81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -875,10 +872,10 @@
         <x:v>crg_core</x:v>
       </x:c>
       <x:c r="F13" s="33" t="str">
-        <x:v>默认与首个唯一上游模块的 npiDefName 精确比较</x:v>
+        <x:v>仅解析、显示并写入报告，当前不参与 PASS/FAIL 判定</x:v>
       </x:c>
       <x:c r="G13" s="33" t="str">
-        <x:v>多驱动或无法解析来源时检查失败</x:v>
+        <x:v>可填写预期来源；当前结果仅供查看，不产生 CRG finding</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="56" customHeight="1">
@@ -889,19 +886,19 @@
         <x:v>RS_CFG_EN</x:v>
       </x:c>
       <x:c r="C14" s="48" t="str">
-        <x:v>条件必填 / 文本</x:v>
+        <x:v>可选 / 文本</x:v>
       </x:c>
       <x:c r="D14" s="47" t="str">
-        <x:v>模块规则声明有同名参数时的假门控标记</x:v>
+        <x:v>RS_CRG_EN 门控参数的兼容标签字段</x:v>
       </x:c>
       <x:c r="E14" s="47" t="str">
         <x:v>假门控</x:v>
       </x:c>
       <x:c r="F14" s="47" t="str">
-        <x:v>按模块规则逐实例检查存在性；参数值为 0 且本列为假门控时通过</x:v>
+        <x:v>规则为 true 时检查参数存在、值为 0 且本列为假门控；规则为 false 时本列不参与判定</x:v>
       </x:c>
       <x:c r="G14" s="47" t="str">
-        <x:v>规则声明无参数时留空；声明有参数时必须填假门控</x:v>
+        <x:v>规则为 true 时必须填假门控；规则为 false 时任意字面内容均可并进入报告</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
@@ -996,7 +993,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a9afd08293f4e57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R896ed16b1d354707"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Allow per-row RS_CFG_EN NA bypass
</commit_message>
<xml_diff>
--- a/examples/RS_Check_Excel_Template.xlsx
+++ b/examples/RS_Check_Excel_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="R5184ee48631e4f5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R3e19f890b83a48b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="Rcbe6515379234868"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="Rde4c61e39d6e4c4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -620,7 +620,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a190cfa1a144a81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fdfa0422fd94af0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -878,7 +878,7 @@
         <x:v>可填写预期来源；当前结果仅供查看，不产生 CRG finding</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="56" customHeight="1">
+    <x:row r="14" ht="72" customHeight="1">
       <x:c r="A14" s="48" t="str">
         <x:v>I</x:v>
       </x:c>
@@ -892,13 +892,13 @@
         <x:v>RS_CRG_EN 门控参数的兼容标签字段</x:v>
       </x:c>
       <x:c r="E14" s="47" t="str">
-        <x:v>假门控</x:v>
+        <x:v>假门控 / NA</x:v>
       </x:c>
       <x:c r="F14" s="47" t="str">
-        <x:v>规则为 true 时检查参数存在、值为 0 且本列为假门控；规则为 false 时本列不参与判定</x:v>
+        <x:v>精确填写 NA 时跳过该行全部 RS_CFG_EN/RS_CRG_EN 检查；否则，规则为 true 时检查参数存在、值为 0 且本列为假门控；规则为 false 时本列不参与判定</x:v>
       </x:c>
       <x:c r="G14" s="47" t="str">
-        <x:v>规则为 true 时必须填假门控；规则为 false 时任意字面内容均可并进入报告</x:v>
+        <x:v>仅精确大写 NA（首尾空白忽略）会跳过；na、N/A 不会。实例匹配、step、clk、rst 等其他检查仍执行</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
@@ -993,7 +993,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R896ed16b1d354707"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14fcb58f4b194e02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add CRG source path mappings
</commit_message>
<xml_diff>
--- a/examples/RS_Check_Excel_Template.xlsx
+++ b/examples/RS_Check_Excel_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="Rcbe6515379234868"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="Rde4c61e39d6e4c4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="Ra834b0a0f5394d76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R8a942a0551d14b91"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -620,7 +620,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fdfa0422fd94af0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27dcdb48e12e404d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -855,7 +855,7 @@
         <x:v>简单信号名可相对 position 填写</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="48" customHeight="1">
+    <x:row r="13" ht="70" customHeight="1">
       <x:c r="A13" s="32" t="str">
         <x:v>H</x:v>
       </x:c>
@@ -866,16 +866,16 @@
         <x:v>是 / 文本</x:v>
       </x:c>
       <x:c r="D13" s="33" t="str">
-        <x:v>该组 clk 连线的预期唯一上游来源模块</x:v>
+        <x:v>该组 clk 预期上游来源模块的简称或完整 RTL 层次路径</x:v>
       </x:c>
       <x:c r="E13" s="33" t="str">
         <x:v>crg_core</x:v>
       </x:c>
       <x:c r="F13" s="33" t="str">
-        <x:v>仅解析、显示并写入报告，当前不参与 PASS/FAIL 判定</x:v>
+        <x:v>先按 config.crg_source_mappings 解析为完整 RTL 路径；仅显示并写入报告，当前不参与 PASS/FAIL 判定</x:v>
       </x:c>
       <x:c r="G13" s="33" t="str">
-        <x:v>可填写预期来源；当前结果仅供查看，不产生 CRG finding</x:v>
+        <x:v>简称需在 GUI CRG Source映射库登记；未命中时按完整路径使用，不产生 CRG finding</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="72" customHeight="1">
@@ -903,7 +903,7 @@
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
       <x:c r="A15" s="37" t="str">
-        <x:v>分组、Position映射与列映射规则</x:v>
+        <x:v>分组、Position/CRG Source映射与列映射规则</x:v>
       </x:c>
       <x:c r="B15" s="37"/>
       <x:c r="C15" s="37"/>
@@ -923,9 +923,9 @@
       <x:c r="F16" s="43"/>
       <x:c r="G16" s="43"/>
     </x:row>
-    <x:row r="17" ht="30" customHeight="1">
+    <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="43" t="str">
-        <x:v>position 可填简写；config.position_mappings 存在同名 key 时解析为对应 RTL 全路径，未命中则兼容原有完整路径。</x:v>
+        <x:v>position 和 CRG_source 均可填简称；分别在 config.position_mappings 和 config.crg_source_mappings 中精确命中后解析为 RTL 全路径，未命中则按完整路径使用。</x:v>
       </x:c>
       <x:c r="B17" s="43"/>
       <x:c r="C17" s="43"/>
@@ -993,7 +993,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14fcb58f4b194e02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9d81ffba3be4c41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add bounded recursive CRG source tracing
</commit_message>
<xml_diff>
--- a/examples/RS_Check_Excel_Template.xlsx
+++ b/examples/RS_Check_Excel_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="Ra834b0a0f5394d76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R8a942a0551d14b91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS_Check" sheetId="1" r:id="R52acc12ce51d482c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R4c304e97f9e94675"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -620,7 +620,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27dcdb48e12e404d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14dd19e446e442cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -872,10 +872,10 @@
         <x:v>crg_core</x:v>
       </x:c>
       <x:c r="F13" s="33" t="str">
-        <x:v>先按 config.crg_source_mappings 解析为完整 RTL 路径；仅显示并写入报告，当前不参与 PASS/FAIL 判定</x:v>
+        <x:v>先按 config.crg_source_mappings 解析为完整 RTL 路径；再从模块规则指定的 RS clk formal 开始，沿上游模块所有 input 有界递归追踪（精确排除 clk、rst_n），并精确匹配完整实例层次路径</x:v>
       </x:c>
       <x:c r="G13" s="33" t="str">
-        <x:v>简称需在 GUI CRG Source映射库登记；未命中时按完整路径使用，不产生 CRG finding</x:v>
+        <x:v>简称需在 GUI CRG Source映射库登记；未命中时按完整路径使用。命中为 pass；未找到、达到 rtl.crg_trace_max_depth 或追踪不可用时产生 CRG warning，但不改变该行其他检查的 PASS/FAIL</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="72" customHeight="1">
@@ -993,7 +993,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9d81ffba3be4c41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0b1be1e93834566"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>